<commit_message>
Add planning docs and commercial dossier
Ultraworked with [Sisyphus](https://github.com/code-yeongyu/oh-my-openagent)

Co-authored-by: Sisyphus <clio-agent@sisyphuslabs.ai>
</commit_message>
<xml_diff>
--- a/docs/planning/creador gantt/GANTT 2026.xlsx
+++ b/docs/planning/creador gantt/GANTT 2026.xlsx
@@ -1680,7 +1680,7 @@
     <row r="22" ht="21" customHeight="1" s="29">
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Driver SPI2 con DMA para ADXL355</t>
+          <t>✅ Driver SPI2 con DMA para ADXL355</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr">
@@ -1904,7 +1904,7 @@
     <row r="26" ht="21" customHeight="1" s="29">
       <c r="B26" s="11" t="inlineStr">
         <is>
-          <t>Suite de Pruebas (Ceedling + Unity, 47 tests)</t>
+          <t>✅ Suite de Pruebas (Ceedling + Unity, 47 tests)</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
@@ -1958,11 +1958,31 @@
       <c r="AF26" s="16" t="n"/>
     </row>
     <row r="27" ht="6" customHeight="1" s="29">
-      <c r="B27" s="17" t="n"/>
-      <c r="C27" s="17" t="n"/>
-      <c r="D27" s="17" t="n"/>
-      <c r="E27" s="17" t="n"/>
-      <c r="F27" s="17" t="n"/>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>✅ Interrupción Wake-on-Motion (WoM) + EXTI</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>Antonio A.</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
       <c r="G27" s="24" t="inlineStr">
         <is>
           <t>T</t>
@@ -1996,16 +2016,32 @@
     <row r="28" ht="22" customHeight="1" s="29">
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>📋 P1 — SISTEMA DE ADQUISICIÓN (Prioridad Alta ~6 meses)</t>
-        </is>
-      </c>
-      <c r="C28" s="10" t="n"/>
-      <c r="D28" s="10" t="n"/>
-      <c r="E28" s="10" t="n"/>
-      <c r="F28" s="10" t="n"/>
+          <t>✅ CLI Extendido (fpu, dma, wom, sensstat, readreg, at, debug)</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Antonio A.</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
+      <c r="F28" s="10" t="inlineStr">
+        <is>
+          <t>Jun 2026</t>
+        </is>
+      </c>
       <c r="G28" s="23" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>T</t>
         </is>
       </c>
       <c r="I28" s="10" t="n"/>
@@ -2036,7 +2072,7 @@
     <row r="29" ht="21" customHeight="1" s="29">
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Adquisición en Tiempo Continuo (sin cortes)</t>
+          <t>🔄 Adquisición en Tiempo Continuo (sin cortes)</t>
         </is>
       </c>
       <c r="C29" s="12" t="inlineStr">
@@ -2046,7 +2082,7 @@
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="E29" s="14" t="inlineStr">
@@ -2092,7 +2128,7 @@
     <row r="30" ht="21" customHeight="1" s="29">
       <c r="B30" s="11" t="inlineStr">
         <is>
-          <t>Optimización DMA (validación + modo burst)</t>
+          <t>✅ Optimización DMA (validación + modo burst)</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
@@ -2102,7 +2138,7 @@
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E30" s="14" t="inlineStr">
@@ -2112,7 +2148,7 @@
       </c>
       <c r="F30" s="14" t="inlineStr">
         <is>
-          <t>Ago 2026</t>
+          <t>Jun 2026</t>
         </is>
       </c>
       <c r="G30" s="24" t="inlineStr">
@@ -2148,7 +2184,7 @@
     <row r="31" ht="21" customHeight="1" s="29">
       <c r="B31" s="11" t="inlineStr">
         <is>
-          <t>Calibración y Caracterización Acelerómetro</t>
+          <t>🔄 Calibración y Caracterización Acelerómetro</t>
         </is>
       </c>
       <c r="C31" s="12" t="inlineStr">
@@ -2158,7 +2194,7 @@
       </c>
       <c r="D31" s="13" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="E31" s="14" t="inlineStr">
@@ -2204,7 +2240,7 @@
     <row r="32" ht="21" customHeight="1" s="29">
       <c r="B32" s="11" t="inlineStr">
         <is>
-          <t>Buffer Local ante pérdida conectividad</t>
+          <t>🔄 Buffer Local ante pérdida conectividad</t>
         </is>
       </c>
       <c r="C32" s="12" t="inlineStr">
@@ -2214,7 +2250,7 @@
       </c>
       <c r="D32" s="13" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="E32" s="14" t="inlineStr">
@@ -2260,7 +2296,7 @@
     <row r="33" ht="21" customHeight="1" s="29">
       <c r="B33" s="11" t="inlineStr">
         <is>
-          <t>Sincronización Horaria (NTP sobre LTE)</t>
+          <t>🔄 Sincronización Horaria (NTP sobre LTE)</t>
         </is>
       </c>
       <c r="C33" s="12" t="inlineStr">
@@ -2270,7 +2306,7 @@
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="E33" s="14" t="inlineStr">
@@ -2316,7 +2352,7 @@
     <row r="34" ht="21" customHeight="1" s="29">
       <c r="B34" s="11" t="inlineStr">
         <is>
-          <t>FPU Enable (configENABLE_FPU=1) + migración</t>
+          <t>✅ FPU Enable (configENABLE_FPU=1) + migración</t>
         </is>
       </c>
       <c r="C34" s="12" t="inlineStr">
@@ -2326,7 +2362,7 @@
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="E34" s="14" t="inlineStr">
@@ -2336,7 +2372,7 @@
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
-          <t>Ago 2026</t>
+          <t>Jun 2026</t>
         </is>
       </c>
       <c r="G34" s="24" t="inlineStr">

</xml_diff>